<commit_message>
Rettelser efter opdeling af model 1+2 og 3, bl.a. i optimization
</commit_message>
<xml_diff>
--- a/Ophold på Kh - Onsdag 2022 1.xlsx
+++ b/Ophold på Kh - Onsdag 2022 1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28816"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dsbintranet-my.sharepoint.com/personal/anluan1805_dsb_dk/Documents/DTU Smarbejde - Speciale &amp; Bachelorprojekter/Data/K22/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carolinehorlykke/Desktop/Bachelor/TTP_bachelor/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B7576F39-5CE4-4CFD-9EE4-20A940F1E41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140F4F3F-03DB-CD43-BE92-5A7696416138}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FInal result" sheetId="2" r:id="rId1"/>
@@ -111,7 +111,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -465,22 +465,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05A74AE-AFAD-4FEF-B14A-A10679167980}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:J112"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="12.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.1640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -512,7 +512,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -544,7 +544,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -576,7 +576,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -597,7 +597,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -629,7 +629,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -661,7 +661,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>10</v>
       </c>
@@ -693,7 +693,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
@@ -725,7 +725,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>10</v>
       </c>
@@ -757,7 +757,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>10</v>
       </c>
@@ -789,7 +789,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
@@ -821,7 +821,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -853,7 +853,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
@@ -885,7 +885,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>10</v>
       </c>
@@ -917,7 +917,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
@@ -949,7 +949,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -981,7 +981,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>10</v>
       </c>
@@ -1013,7 +1013,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>10</v>
       </c>
@@ -1045,7 +1045,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>10</v>
       </c>
@@ -1077,7 +1077,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>10</v>
       </c>
@@ -1098,7 +1098,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>10</v>
       </c>
@@ -1130,7 +1130,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>10</v>
       </c>
@@ -1162,7 +1162,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>10</v>
       </c>
@@ -1194,7 +1194,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>10</v>
       </c>
@@ -1226,7 +1226,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>10</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>10</v>
       </c>
@@ -1290,7 +1290,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>10</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>10</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>10</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>10</v>
       </c>
@@ -1418,7 +1418,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>10</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>10</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>10</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>10</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>10</v>
       </c>
@@ -1578,7 +1578,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>10</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>10</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>10</v>
       </c>
@@ -1674,7 +1674,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>10</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>10</v>
       </c>
@@ -1727,7 +1727,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>10</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>10</v>
       </c>
@@ -1780,7 +1780,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>10</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>10</v>
       </c>
@@ -1844,7 +1844,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>10</v>
       </c>
@@ -1876,7 +1876,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>10</v>
       </c>
@@ -1908,7 +1908,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="47" spans="1:10">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>10</v>
       </c>
@@ -1940,7 +1940,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="48" spans="1:10">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>10</v>
       </c>
@@ -1972,7 +1972,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>10</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>10</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>10</v>
       </c>
@@ -2068,7 +2068,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>10</v>
       </c>
@@ -2100,7 +2100,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>10</v>
       </c>
@@ -2132,7 +2132,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>10</v>
       </c>
@@ -2153,7 +2153,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>10</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>10</v>
       </c>
@@ -2217,7 +2217,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="57" spans="1:10">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>10</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:10">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>10</v>
       </c>
@@ -2281,7 +2281,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="59" spans="1:10">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>10</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>10</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>10</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>10</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>10</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>10</v>
       </c>
@@ -2473,7 +2473,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>10</v>
       </c>
@@ -2505,7 +2505,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>10</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>10</v>
       </c>
@@ -2558,7 +2558,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>10</v>
       </c>
@@ -2590,7 +2590,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>10</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="70" spans="1:10">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>10</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>10</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>10</v>
       </c>
@@ -2707,7 +2707,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="73" spans="1:10">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>10</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="74" spans="1:10">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>10</v>
       </c>
@@ -2771,7 +2771,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>10</v>
       </c>
@@ -2803,7 +2803,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="76" spans="1:10">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>10</v>
       </c>
@@ -2835,7 +2835,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="77" spans="1:10">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>10</v>
       </c>
@@ -2867,7 +2867,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="78" spans="1:10">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>10</v>
       </c>
@@ -2899,7 +2899,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="79" spans="1:10">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>10</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="80" spans="1:10">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>10</v>
       </c>
@@ -2963,7 +2963,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="1:10">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>10</v>
       </c>
@@ -2995,7 +2995,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:10">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>10</v>
       </c>
@@ -3027,7 +3027,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:10">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>10</v>
       </c>
@@ -3059,7 +3059,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:10">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>10</v>
       </c>
@@ -3091,7 +3091,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="85" spans="1:10">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>10</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="86" spans="1:10">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>10</v>
       </c>
@@ -3155,7 +3155,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:10">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>10</v>
       </c>
@@ -3187,7 +3187,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="88" spans="1:10">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>10</v>
       </c>
@@ -3219,7 +3219,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:10">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>10</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="1:10">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>10</v>
       </c>
@@ -3283,7 +3283,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="91" spans="1:10">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>10</v>
       </c>
@@ -3315,7 +3315,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:10">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>10</v>
       </c>
@@ -3347,7 +3347,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="93" spans="1:10">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>10</v>
       </c>
@@ -3379,7 +3379,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="94" spans="1:10">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>10</v>
       </c>
@@ -3411,7 +3411,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="95" spans="1:10">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>10</v>
       </c>
@@ -3443,7 +3443,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="96" spans="1:10">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>10</v>
       </c>
@@ -3475,7 +3475,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="97" spans="1:10">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>10</v>
       </c>
@@ -3507,7 +3507,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:10">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>10</v>
       </c>
@@ -3539,7 +3539,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="99" spans="1:10">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>10</v>
       </c>
@@ -3571,7 +3571,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="100" spans="1:10">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>10</v>
       </c>
@@ -3603,7 +3603,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:10">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>10</v>
       </c>
@@ -3635,7 +3635,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="102" spans="1:10">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>10</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="103" spans="1:10">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>10</v>
       </c>
@@ -3699,7 +3699,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104" spans="1:10">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>10</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:10">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>10</v>
       </c>
@@ -3763,7 +3763,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="1:10">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>10</v>
       </c>
@@ -3795,7 +3795,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="107" spans="1:10">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>10</v>
       </c>
@@ -3827,7 +3827,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="108" spans="1:10">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>10</v>
       </c>
@@ -3859,7 +3859,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="109" spans="1:10">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>10</v>
       </c>
@@ -3880,7 +3880,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="110" spans="1:10">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>10</v>
       </c>
@@ -3912,7 +3912,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="111" spans="1:10">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>10</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="112" spans="1:10">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>10</v>
       </c>
@@ -3988,5 +3988,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF8B71D7-FEF4-4CE3-BFC8-A514080C30BF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CF8B71D7-FEF4-4CE3-BFC8-A514080C30BF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>